<commit_message>
Reorganize repo: Task 1 deliverables into Task_1_EDA/, add repo-level README
</commit_message>
<xml_diff>
--- a/Delinquency_prediction_dataset.xlsx
+++ b/Delinquency_prediction_dataset.xlsx
@@ -1,39 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/AYoung/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/TTran/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2E70A54-EF18-1346-BD1B-8D1FBB191312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E750397F-8D62-0948-8D40-5D563B1F8FD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16300" xr2:uid="{B456ABAB-9710-1A41-9AAD-930C444190E8}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16940" xr2:uid="{B456ABAB-9710-1A41-9AAD-930C444190E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Delinquency_prediction_dataset" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5019" uniqueCount="538">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="5019" uniqueCount="538">
   <si>
     <t>Customer_ID</t>
   </si>
@@ -1652,7 +1644,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -1972,15 +1964,15 @@
   </fills>
   <borders count="10">
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="thick">
         <color theme="4"/>
@@ -1988,8 +1980,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="thick">
         <color theme="4" tint="0.499984740745262"/>
@@ -1997,8 +1989,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="medium">
         <color theme="4" tint="0.39997558519241921"/>
@@ -2006,12 +1998,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
+      </start>
+      <end style="thin">
         <color rgb="FF7F7F7F"/>
-      </right>
+      </end>
       <top style="thin">
         <color rgb="FF7F7F7F"/>
       </top>
@@ -2021,12 +2013,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
+      </start>
+      <end style="thin">
         <color rgb="FF3F3F3F"/>
-      </right>
+      </end>
       <top style="thin">
         <color rgb="FF3F3F3F"/>
       </top>
@@ -2036,8 +2028,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
@@ -2045,12 +2037,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
+      <start style="double">
         <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
+      </start>
+      <end style="double">
         <color rgb="FF3F3F3F"/>
-      </right>
+      </end>
       <top style="double">
         <color rgb="FF3F3F3F"/>
       </top>
@@ -2060,12 +2052,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
+      </start>
+      <end style="thin">
         <color rgb="FFB2B2B2"/>
-      </right>
+      </end>
       <top style="thin">
         <color rgb="FFB2B2B2"/>
       </top>
@@ -2075,8 +2067,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -2191,7 +2183,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://purl.oclc.org/ooxml/drawingml/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2344,25 +2336,25 @@
         </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0">
+            <a:gs pos="0%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:lumMod val="110%"/>
+                <a:satMod val="105%"/>
+                <a:tint val="67%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="50%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:lumMod val="105%"/>
+                <a:satMod val="103%"/>
+                <a:tint val="73%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
+            <a:gs pos="100%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:lumMod val="105%"/>
+                <a:satMod val="109%"/>
+                <a:tint val="81%"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -2370,25 +2362,25 @@
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0">
+            <a:gs pos="0%">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:satMod val="103%"/>
+                <a:lumMod val="102%"/>
+                <a:tint val="94%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="50%">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:satMod val="110%"/>
+                <a:lumMod val="100%"/>
+                <a:shade val="100%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
+            <a:gs pos="100%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:lumMod val="99%"/>
+                <a:satMod val="120%"/>
+                <a:shade val="78%"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -2401,21 +2393,21 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter lim="800%"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter lim="800%"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter lim="800%"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -2429,7 +2421,7 @@
           <a:effectLst>
             <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="63%"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -2441,32 +2433,32 @@
         </a:solidFill>
         <a:solidFill>
           <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
+            <a:tint val="95%"/>
+            <a:satMod val="170%"/>
           </a:schemeClr>
         </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0">
+            <a:gs pos="0%">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="93%"/>
+                <a:satMod val="150%"/>
+                <a:shade val="98%"/>
+                <a:lumMod val="102%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="50%">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="98%"/>
+                <a:satMod val="130%"/>
+                <a:shade val="90%"/>
+                <a:lumMod val="103%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
+            <a:gs pos="100%">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="63%"/>
+                <a:satMod val="120%"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -2506,7 +2498,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCFB9B7-0511-9A41-B96E-08EFA2105853}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCFB9B7-0511-9A41-B96E-08EFA2105853}">
   <dimension ref="A1:S501"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>